<commit_message>
added metric calculation data
</commit_message>
<xml_diff>
--- a/Annotation Data/Test Set Annotations - Coder 2.xlsx
+++ b/Annotation Data/Test Set Annotations - Coder 2.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Computer Science\AnanyaSingh_Project_Data\Annotation Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Computer Science\AnanyaSingh_Project_Data\RP_Project\Annotation Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F1096962-E973-4AB7-80C9-23FAF6720D13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8A86826-59EF-4EC9-8DA2-B2C62043D048}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="5" xr2:uid="{0C98FBDC-CD59-41DB-9754-1C3037231F78}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="4" activeTab="5" xr2:uid="{0C98FBDC-CD59-41DB-9754-1C3037231F78}"/>
   </bookViews>
   <sheets>
     <sheet name="Facial Recognition Technology" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="Predictive Policing" sheetId="3" r:id="rId3"/>
     <sheet name="Extend CCTV Footage Retention" sheetId="4" r:id="rId4"/>
     <sheet name="Biometric Border Control" sheetId="5" r:id="rId5"/>
-    <sheet name="Sheet6" sheetId="6" r:id="rId6"/>
+    <sheet name="Drone" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -1161,7 +1161,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="409.6" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" ht="124.8" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>43</v>
       </c>
@@ -1178,7 +1178,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="409.6" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" ht="109.2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>37</v>
       </c>
@@ -1195,7 +1195,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="409.6" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" ht="109.2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>50</v>
       </c>
@@ -1246,7 +1246,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="409.6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" ht="187.2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>54</v>
       </c>
@@ -1260,7 +1260,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="409.6" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" ht="187.2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>57</v>
       </c>
@@ -1274,7 +1274,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="187.2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" ht="46.8" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>60</v>
       </c>
@@ -1288,7 +1288,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="312" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" ht="78" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>60</v>
       </c>
@@ -1305,7 +1305,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="409.6" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" ht="109.2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>64</v>
       </c>
@@ -1322,7 +1322,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="409.6" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" ht="109.2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>67</v>
       </c>
@@ -1339,7 +1339,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="312" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" ht="62.4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>60</v>
       </c>
@@ -1418,7 +1418,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="374.4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" ht="124.8" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>75</v>
       </c>
@@ -1432,7 +1432,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="234" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" ht="78" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>75</v>
       </c>
@@ -1446,7 +1446,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="156" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" ht="62.4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>81</v>
       </c>
@@ -1474,7 +1474,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="234" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" ht="93.6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>72</v>
       </c>
@@ -1488,7 +1488,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="374.4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" ht="140.4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>75</v>
       </c>
@@ -1536,7 +1536,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="249.6" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" ht="93.6" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>81</v>
       </c>
@@ -1553,7 +1553,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="265.2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" ht="109.2" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>81</v>
       </c>
@@ -1567,7 +1567,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="280.8" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" ht="109.2" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>89</v>
       </c>
@@ -1646,7 +1646,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="187.2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" ht="62.4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>104</v>
       </c>
@@ -1660,7 +1660,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="218.4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" ht="62.4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>98</v>
       </c>
@@ -1674,7 +1674,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="343.2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" ht="93.6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>98</v>
       </c>
@@ -1691,7 +1691,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="280.8" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" ht="78" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>111</v>
       </c>
@@ -1705,7 +1705,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="280.8" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" ht="78" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>101</v>
       </c>
@@ -1719,7 +1719,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="358.8" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" ht="109.2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>104</v>
       </c>
@@ -1733,7 +1733,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="409.6" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" ht="156" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>111</v>
       </c>
@@ -1747,7 +1747,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="140.4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" ht="46.8" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>101</v>
       </c>
@@ -1764,7 +1764,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="187.2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" ht="62.4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>111</v>
       </c>
@@ -1781,7 +1781,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="358.8" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" ht="93.6" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>111</v>
       </c>
@@ -1875,7 +1875,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="390" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" ht="124.8" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>131</v>
       </c>
@@ -1889,7 +1889,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="171.6" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" ht="62.4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>132</v>
       </c>
@@ -1903,7 +1903,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="202.8" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" ht="78" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>132</v>
       </c>
@@ -1917,7 +1917,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="280.8" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" ht="78" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>60</v>
       </c>
@@ -1948,7 +1948,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="390" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" ht="140.4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>129</v>
       </c>
@@ -1965,7 +1965,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="280.8" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" ht="78" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>132</v>
       </c>
@@ -1996,6 +1996,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A3067A853EBED448818D481A45977CAD" ma:contentTypeVersion="13" ma:contentTypeDescription="Een nieuw document maken." ma:contentTypeScope="" ma:versionID="800a9b9b73224d82f19595a45945cab9">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="9a36658d-ac49-47b7-a59e-e908f59ad619" xmlns:ns4="4e95ffdb-565a-4842-9a76-98f37fb297b0" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2f792393693ac5ebddb1ed28a5e00ea0" ns3:_="" ns4:_="">
     <xsd:import namespace="9a36658d-ac49-47b7-a59e-e908f59ad619"/>
@@ -2216,15 +2225,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -2234,6 +2234,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{021767AC-03A6-4D42-A48A-ED980B2D57B2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0674AE1C-C88D-447F-8509-7271D748C21A}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2248,14 +2256,6 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{021767AC-03A6-4D42-A48A-ED980B2D57B2}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>